<commit_message>
Added gerbers of PDMS v4.3, assembly docs, modified DNP parameters
</commit_message>
<xml_diff>
--- a/PCB/PDMS/pdms/BOMS_DOCS/pdms_v4.3_bom.xlsx
+++ b/PCB/PDMS/pdms/BOMS_DOCS/pdms_v4.3_bom.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karol\Documents\GitHub\PDM\PCB\PDMS\pdms\BOMS_DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52664F18-AB97-4AFA-9B24-603C03FBD50B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4553BC7B-9F2E-460A-831E-DAA872E720ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="51870" windowHeight="21420" xr2:uid="{63C5BD05-1EB6-42C1-8154-EDFC7CCC6969}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{63C5BD05-1EB6-42C1-8154-EDFC7CCC6969}"/>
   </bookViews>
   <sheets>
     <sheet name="pdms_v4 3_bom" sheetId="2" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">'pdms_v4 3_bom'!$B$1:$G$116</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2058,7 +2059,7 @@
         <v>10</v>
       </c>
       <c r="H14" s="1">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2665,7 +2666,7 @@
         <v>10</v>
       </c>
       <c r="H38" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>